<commit_message>
Fix resource plan source headers
</commit_message>
<xml_diff>
--- a/data/contractors/derived-4700134228/sources/equipment_plan.xlsx
+++ b/data/contractors/derived-4700134228/sources/equipment_plan.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Техника" sheetId="1" r:id="R77673fad74b547f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="План по месяцам" sheetId="2" r:id="R71aaee4774014412"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Техника" sheetId="1" r:id="R83bddf88ba634293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="План по месяцам" sheetId="2" r:id="R1fd0028735484b57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -328,22 +328,22 @@
         <x:v>Категория</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>KQ</x:v>
+        <x:v>Тип</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
-        <x:v>Дисциплина</x:v>
+        <x:v>Техника</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
         <x:v>Работа</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Персонал</x:v>
+        <x:v>KQ</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str">
+        <x:v>Дисциплина</x:v>
+      </x:c>
+      <x:c r="L4" s="6" t="str">
         <x:v>ИТОГО</x:v>
-      </x:c>
-      <x:c r="L4" s="6" t="str">
-        <x:v>Всего дней/машин</x:v>
       </x:c>
       <x:c r="M4" s="11" t="n">
         <x:v>45992.5</x:v>

</xml_diff>